<commit_message>
Aligned all I/O buffers for improved throughput.
</commit_message>
<xml_diff>
--- a/doc/pcg64dxsm-performance.xlsx
+++ b/doc/pcg64dxsm-performance.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="15">
   <si>
     <t>PCG64DXSM</t>
   </si>
@@ -53,6 +53,15 @@
   <si>
     <t>ST</t>
   </si>
+  <si>
+    <t>Ubuntu 24.04 (x64)</t>
+  </si>
+  <si>
+    <t>macOS 26.4 (arm64)</t>
+  </si>
+  <si>
+    <t>Windows 11 (x64)</t>
+  </si>
 </sst>
 </file>
 
@@ -61,7 +70,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -82,6 +91,20 @@
       <color theme="1"/>
       <name val="Lucida Console"/>
       <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -133,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -152,6 +175,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,270 +486,330 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="B4">
         <v>3351.4</v>
       </c>
-      <c r="C2">
+      <c r="C4">
         <v>3571.5</v>
       </c>
-      <c r="D2">
+      <c r="D4">
         <v>3091.6</v>
       </c>
-      <c r="E2">
+      <c r="E4">
         <v>2854.4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3">
+      <c r="B5">
         <v>3855.3</v>
       </c>
-      <c r="C3">
+      <c r="C5">
         <v>4320.8999999999996</v>
       </c>
-      <c r="D3">
+      <c r="D5">
         <v>3607.2</v>
       </c>
-      <c r="E3">
+      <c r="E5">
         <v>3407.1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>3361.8</v>
-      </c>
-      <c r="C6">
-        <v>3908.6</v>
-      </c>
-      <c r="D6">
-        <v>4266.1000000000004</v>
-      </c>
-      <c r="E6">
-        <v>4074.6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7">
-        <v>3465.8</v>
-      </c>
-      <c r="C7">
-        <v>3996.8</v>
-      </c>
-      <c r="D7">
-        <v>4414.8999999999996</v>
-      </c>
-      <c r="E7">
-        <v>4097.3999999999996</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B8">
-        <v>3471.4</v>
+        <v>3361.8</v>
       </c>
       <c r="C8">
-        <v>4127.2</v>
+        <v>3908.6</v>
       </c>
       <c r="D8">
-        <v>4460.8</v>
+        <v>4266.1000000000004</v>
       </c>
       <c r="E8">
-        <v>4193.6000000000004</v>
+        <v>4074.6</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <v>3465.8</v>
+      </c>
+      <c r="C9">
+        <v>3996.8</v>
+      </c>
+      <c r="D9">
+        <v>4414.8999999999996</v>
+      </c>
+      <c r="E9">
+        <v>4097.3999999999996</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>3471.4</v>
+      </c>
+      <c r="C10">
+        <v>4127.2</v>
+      </c>
+      <c r="D10">
+        <v>4460.8</v>
+      </c>
+      <c r="E10">
+        <v>4193.6000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B9">
+      <c r="B11">
         <v>3504.2</v>
       </c>
-      <c r="C9">
+      <c r="C11">
         <v>4056.8</v>
       </c>
-      <c r="D9">
+      <c r="D11">
         <v>4536.7</v>
       </c>
-      <c r="E9">
+      <c r="E11">
         <v>4228.8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B10">
+      <c r="B12">
         <v>3510.2</v>
       </c>
-      <c r="C10">
+      <c r="C12">
         <v>4096.6000000000004</v>
       </c>
-      <c r="D10">
+      <c r="D12">
         <v>4499.8</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E12" s="6">
         <v>4174</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13">
-        <v>3397.6</v>
-      </c>
-      <c r="C13" s="3">
-        <v>3947</v>
-      </c>
-      <c r="D13" s="3">
-        <v>4302</v>
-      </c>
-      <c r="E13" s="3">
-        <v>3996</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14">
-        <v>3348.4</v>
-      </c>
-      <c r="C14">
-        <v>3944.1</v>
-      </c>
-      <c r="D14" s="3">
-        <v>4384</v>
-      </c>
-      <c r="E14">
-        <v>4082.7</v>
       </c>
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B15">
-        <v>3468.3</v>
-      </c>
-      <c r="C15">
-        <v>3983.9</v>
-      </c>
-      <c r="D15">
-        <v>4435.5</v>
-      </c>
-      <c r="E15" s="4">
-        <v>4155.3</v>
+        <v>3397.6</v>
+      </c>
+      <c r="C15" s="3">
+        <v>3947</v>
+      </c>
+      <c r="D15" s="3">
+        <v>4302</v>
+      </c>
+      <c r="E15" s="3">
+        <v>3996</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16">
+        <v>3348.4</v>
+      </c>
+      <c r="C16">
+        <v>3944.1</v>
+      </c>
+      <c r="D16" s="3">
+        <v>4384</v>
+      </c>
+      <c r="E16">
+        <v>4082.7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17">
+        <v>3468.3</v>
+      </c>
+      <c r="C17">
+        <v>3983.9</v>
+      </c>
+      <c r="D17">
+        <v>4435.5</v>
+      </c>
+      <c r="E17" s="4">
+        <v>4155.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B16">
+      <c r="B18">
         <v>3509.5</v>
       </c>
-      <c r="C16">
+      <c r="C18">
         <v>3978.3</v>
       </c>
-      <c r="D16">
+      <c r="D18">
         <v>4462.1000000000004</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E18" s="3">
         <v>4159</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B17">
+      <c r="B19">
         <v>3503.6</v>
       </c>
-      <c r="C17">
+      <c r="C19">
         <v>4057.4</v>
       </c>
-      <c r="D17">
+      <c r="D19">
         <v>4538.2</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E19" s="4">
         <v>4098.7</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B7:E7 C8">
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9:E9 C10">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 C10">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E10">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -729,7 +821,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B14:E14">
+  <conditionalFormatting sqref="B15:E17 F14">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -741,7 +833,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E7 C8">
+  <conditionalFormatting sqref="B8:E11">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -753,7 +845,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E14">
+  <conditionalFormatting sqref="B15:E18">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -765,55 +857,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E8">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E15 F14">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E9">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E16">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E10">
+  <conditionalFormatting sqref="B8:E12">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -825,7 +869,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E17">
+  <conditionalFormatting sqref="B15:E19">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -837,7 +881,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:E2">
+  <conditionalFormatting sqref="B4:E4">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -849,7 +893,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:E3">
+  <conditionalFormatting sqref="B5:E5">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -868,175 +912,282 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="B4">
         <v>2826.9</v>
       </c>
-      <c r="C2">
+      <c r="C4">
         <v>3235.8</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D4" s="3">
         <v>2945</v>
       </c>
-      <c r="E2">
+      <c r="E4">
         <v>2852.8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3">
+      <c r="B5">
         <v>3572.4</v>
       </c>
-      <c r="C3">
+      <c r="C5">
         <v>4015.7</v>
       </c>
-      <c r="D3">
+      <c r="D5">
         <v>3625.3</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E5" s="4">
         <v>3416.8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7">
-        <v>3671.7</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8">
-        <v>3670.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>3671.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>3655.1</v>
+      </c>
+      <c r="D10">
+        <v>3707.1</v>
+      </c>
+      <c r="E10">
+        <v>3758.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D9">
+      <c r="D11">
         <v>3671.4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="E12" s="6"/>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D14" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="3">
-        <v>5032.6000000000004</v>
       </c>
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15">
-        <v>5037.6000000000004</v>
-      </c>
-      <c r="E15" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3">
+        <v>5032.6000000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="4">
+        <v>4959.8</v>
+      </c>
+      <c r="D17">
+        <v>5042.8</v>
+      </c>
+      <c r="E17">
+        <v>4984.6000000000004</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D16">
+      <c r="D18">
         <v>5035.5</v>
       </c>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E17" s="4"/>
+      <c r="E19" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B7:E7 C8">
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9:E9">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 B10:D10">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16 F14 B17:D17">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 B11:E11 B10:D10">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16 B18:E18 B17:D17">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -1048,19 +1199,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B14:E14">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E7 C8">
+  <conditionalFormatting sqref="B8:E9 B11:E12 B10:D10">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16 B18:E19 B17:D17">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1072,55 +1223,43 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E14">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E8">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E15 F14">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E9">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E16">
+  <conditionalFormatting sqref="B4:E4">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:E5">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E19">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:E11">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -1132,19 +1271,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E10">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E17">
+  <conditionalFormatting sqref="B4:E5">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E12">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1156,179 +1295,284 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:E2">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:E3">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3">
-        <v>2540</v>
-      </c>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="B4" s="3">
+        <v>1868</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2689</v>
+      </c>
+      <c r="D4" s="3">
+        <v>3412</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C3">
-        <v>2927.6</v>
-      </c>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="B5">
+        <v>2148.3000000000002</v>
+      </c>
+      <c r="C5">
+        <v>3012.6</v>
+      </c>
+      <c r="D5">
+        <v>3943.1</v>
+      </c>
+      <c r="E5" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8">
-        <v>5627.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>5648.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>4886.8</v>
+      </c>
+      <c r="D10">
+        <v>5644.2</v>
+      </c>
+      <c r="E10">
+        <v>5655.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="D11">
+        <v>5673.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="E12" s="6"/>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D14" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="3"/>
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" s="3">
-        <v>6929</v>
-      </c>
-      <c r="E15" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3">
+        <v>6675.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>4859.3</v>
+      </c>
+      <c r="D17" s="3">
+        <v>7126.5</v>
+      </c>
+      <c r="E17" s="4">
+        <v>6681.1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="D18" s="3">
+        <v>6922</v>
+      </c>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E17" s="4"/>
+      <c r="E19" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B7:E7 C8">
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9:E9 C10">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 C10">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E10">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E17 F14">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E11">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E18">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -1340,7 +1584,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B14:E14">
+  <conditionalFormatting sqref="B8:E12">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E19">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1352,43 +1608,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E7 C8">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E14">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E8">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E15 F14">
+  <conditionalFormatting sqref="B4:E4">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:E5">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:E5">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -1400,31 +1644,43 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E9">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E16">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:E10">
+  <conditionalFormatting sqref="C17:E17">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10:E10">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:E11">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16:E18">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1436,43 +1692,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E17">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:E2">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:E3">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added support for parameters '--st' and '--mt' to the benchmarking program.
</commit_message>
<xml_diff>
--- a/doc/pcg64dxsm-performance.xlsx
+++ b/doc/pcg64dxsm-performance.xlsx
@@ -526,10 +526,10 @@
         <v>3351.4</v>
       </c>
       <c r="C4">
-        <v>3571.5</v>
+        <v>3488.6</v>
       </c>
       <c r="D4">
-        <v>3091.6</v>
+        <v>2960.4</v>
       </c>
       <c r="E4">
         <v>2854.4</v>
@@ -542,11 +542,11 @@
       <c r="B5">
         <v>3855.3</v>
       </c>
-      <c r="C5">
-        <v>4320.8999999999996</v>
+      <c r="C5" s="3">
+        <v>4199</v>
       </c>
       <c r="D5">
-        <v>3607.2</v>
+        <v>3622.2</v>
       </c>
       <c r="E5">
         <v>3407.1</v>
@@ -614,7 +614,7 @@
         <v>4127.2</v>
       </c>
       <c r="D10">
-        <v>4460.8</v>
+        <v>4460.2</v>
       </c>
       <c r="E10">
         <v>4193.6000000000004</v>
@@ -664,7 +664,7 @@
       <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -716,8 +716,8 @@
       <c r="C17">
         <v>3983.9</v>
       </c>
-      <c r="D17">
-        <v>4435.5</v>
+      <c r="D17" s="3">
+        <v>4472.2</v>
       </c>
       <c r="E17" s="4">
         <v>4155.3</v>

</xml_diff>

<commit_message>
Slightly tweak ST buffer size for the Windows platform.
</commit_message>
<xml_diff>
--- a/doc/pcg64dxsm-performance.xlsx
+++ b/doc/pcg64dxsm-performance.xlsx
@@ -9,14 +9,15 @@
   <sheets>
     <sheet name="Ubuntu 24.04 (x64)" sheetId="1" r:id="rId1"/>
     <sheet name="macOS 26.4 (arm64)" sheetId="4" r:id="rId2"/>
-    <sheet name="Windows 11 (x64)" sheetId="5" r:id="rId3"/>
+    <sheet name="Windows 11 (x64) (NB)" sheetId="5" r:id="rId3"/>
+    <sheet name="Windows 11 (x64) (PC)" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="16">
   <si>
     <t>PCG64DXSM</t>
   </si>
@@ -62,6 +63,9 @@
   <si>
     <t>Windows 11 (x64)</t>
   </si>
+  <si>
+    <t>8 KB</t>
+  </si>
 </sst>
 </file>
 
@@ -70,7 +74,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,6 +110,26 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -115,7 +139,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -152,11 +176,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -179,7 +214,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -493,28 +543,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -523,33 +576,39 @@
         <v>0</v>
       </c>
       <c r="B4">
-        <v>3351.4</v>
+        <v>3025.6</v>
       </c>
       <c r="C4">
-        <v>3488.6</v>
+        <v>3548.3</v>
       </c>
       <c r="D4">
-        <v>2960.4</v>
+        <v>4018.4</v>
       </c>
       <c r="E4">
-        <v>2854.4</v>
+        <v>3061.8</v>
+      </c>
+      <c r="F4">
+        <v>2874.5</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B5">
-        <v>3855.3</v>
-      </c>
-      <c r="C5" s="3">
-        <v>4199</v>
-      </c>
-      <c r="D5">
-        <v>3622.2</v>
+      <c r="B5" s="3">
+        <v>3935</v>
+      </c>
+      <c r="C5">
+        <v>4247.5</v>
+      </c>
+      <c r="D5" s="3">
+        <v>4570.8</v>
       </c>
       <c r="E5">
-        <v>3407.1</v>
+        <v>3777.3</v>
+      </c>
+      <c r="F5" s="3">
+        <v>3400</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -562,7 +621,7 @@
       <c r="C7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="12" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -574,50 +633,50 @@
         <v>1</v>
       </c>
       <c r="B8">
-        <v>3361.8</v>
+        <v>3378.6</v>
       </c>
       <c r="C8">
-        <v>3908.6</v>
+        <v>4206.8</v>
       </c>
       <c r="D8">
-        <v>4266.1000000000004</v>
+        <v>4062.5</v>
       </c>
       <c r="E8">
-        <v>4074.6</v>
+        <v>4165.1000000000004</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="14" t="s">
         <v>2</v>
       </c>
       <c r="B9">
-        <v>3465.8</v>
+        <v>3547.5</v>
       </c>
       <c r="C9">
-        <v>3996.8</v>
+        <v>4246.6000000000004</v>
       </c>
       <c r="D9">
-        <v>4414.8999999999996</v>
+        <v>4536.5</v>
       </c>
       <c r="E9">
-        <v>4097.3999999999996</v>
+        <v>4269.8</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="15" t="s">
         <v>3</v>
       </c>
       <c r="B10">
-        <v>3471.4</v>
+        <v>3703.7</v>
       </c>
       <c r="C10">
-        <v>4127.2</v>
+        <v>4263.7</v>
       </c>
       <c r="D10">
-        <v>4460.2</v>
+        <v>4461.3999999999996</v>
       </c>
       <c r="E10">
-        <v>4193.6000000000004</v>
+        <v>4393.8999999999996</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -625,34 +684,23 @@
         <v>4</v>
       </c>
       <c r="B11">
-        <v>3504.2</v>
+        <v>3637.1</v>
       </c>
       <c r="C11">
-        <v>4056.8</v>
+        <v>4194</v>
       </c>
       <c r="D11">
-        <v>4536.7</v>
-      </c>
-      <c r="E11">
-        <v>4228.8</v>
+        <v>4668.8</v>
+      </c>
+      <c r="E11" s="4">
+        <v>4333.2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B12">
-        <v>3510.2</v>
-      </c>
-      <c r="C12">
-        <v>4096.6000000000004</v>
-      </c>
-      <c r="D12">
-        <v>4499.8</v>
-      </c>
-      <c r="E12" s="6">
-        <v>4174</v>
-      </c>
+      <c r="E12" s="6"/>
     </row>
     <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
@@ -664,7 +712,7 @@
       <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="12" t="s">
         <v>7</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -677,50 +725,50 @@
         <v>1</v>
       </c>
       <c r="B15">
-        <v>3397.6</v>
+        <v>3288.8</v>
       </c>
       <c r="C15" s="3">
-        <v>3947</v>
+        <v>4062.5</v>
       </c>
       <c r="D15" s="3">
-        <v>4302</v>
+        <v>4465.8999999999996</v>
       </c>
       <c r="E15" s="3">
-        <v>3996</v>
+        <v>4149.7</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="14" t="s">
         <v>2</v>
       </c>
       <c r="B16">
-        <v>3348.4</v>
+        <v>3574.1</v>
       </c>
       <c r="C16">
-        <v>3944.1</v>
+        <v>3992.1</v>
       </c>
       <c r="D16" s="3">
-        <v>4384</v>
+        <v>4827.1000000000004</v>
       </c>
       <c r="E16">
-        <v>4082.7</v>
+        <v>4183.2</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="15" t="s">
         <v>3</v>
       </c>
       <c r="B17">
-        <v>3468.3</v>
+        <v>3756.7</v>
       </c>
       <c r="C17">
-        <v>3983.9</v>
+        <v>4351.6000000000004</v>
       </c>
       <c r="D17" s="3">
-        <v>4472.2</v>
+        <v>4560.3</v>
       </c>
       <c r="E17" s="4">
-        <v>4155.3</v>
+        <v>4276.8</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -728,41 +776,30 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>3509.5</v>
-      </c>
-      <c r="C18">
-        <v>3978.3</v>
+        <v>3643.3</v>
+      </c>
+      <c r="C18" s="3">
+        <v>4314</v>
       </c>
       <c r="D18">
-        <v>4462.1000000000004</v>
+        <v>4907.7</v>
       </c>
       <c r="E18" s="3">
-        <v>4159</v>
+        <v>4275.8999999999996</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B19">
-        <v>3503.6</v>
-      </c>
-      <c r="C19">
-        <v>4057.4</v>
-      </c>
-      <c r="D19">
-        <v>4538.2</v>
-      </c>
-      <c r="E19" s="4">
-        <v>4098.7</v>
-      </c>
+      <c r="E19" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="B9:E9 C10">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -774,7 +811,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:E16">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -786,7 +823,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:E9 C10">
-    <cfRule type="colorScale" priority="14">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -798,7 +835,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:E16">
-    <cfRule type="colorScale" priority="13">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -810,7 +847,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:E10">
-    <cfRule type="colorScale" priority="12">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -822,6 +859,42 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:E17 F14">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E11">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E18">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E12">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -833,7 +906,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E11">
+  <conditionalFormatting sqref="B15:E19">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -845,7 +918,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E18">
+  <conditionalFormatting sqref="C4:F4">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -857,44 +930,32 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E12">
+  <conditionalFormatting sqref="C5:F5">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:F4">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:F5">
     <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E19">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E4">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:E5">
-    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -919,28 +980,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -949,16 +1013,19 @@
         <v>0</v>
       </c>
       <c r="B4">
-        <v>2826.9</v>
+        <v>1855.5</v>
       </c>
       <c r="C4">
-        <v>3235.8</v>
-      </c>
-      <c r="D4" s="3">
-        <v>2945</v>
-      </c>
-      <c r="E4">
-        <v>2852.8</v>
+        <v>2813.3</v>
+      </c>
+      <c r="D4">
+        <v>3259.4</v>
+      </c>
+      <c r="E4" s="3">
+        <v>3083.6</v>
+      </c>
+      <c r="F4">
+        <v>3010.7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -966,16 +1033,19 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>3572.4</v>
+        <v>3299.7</v>
       </c>
       <c r="C5">
-        <v>4015.7</v>
-      </c>
-      <c r="D5">
-        <v>3625.3</v>
-      </c>
-      <c r="E5" s="4">
-        <v>3416.8</v>
+        <v>3610.2</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3966.89</v>
+      </c>
+      <c r="E5">
+        <v>3723.6</v>
+      </c>
+      <c r="F5" s="4">
+        <v>3548.5</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -999,42 +1069,86 @@
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B8" s="3">
+        <v>3879.1</v>
+      </c>
+      <c r="C8" s="3">
+        <v>3700.6</v>
+      </c>
+      <c r="D8" s="3">
+        <v>3704.4</v>
+      </c>
+      <c r="E8" s="3">
+        <v>3767.1</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D9">
-        <v>3671.7</v>
+      <c r="B9" s="3">
+        <v>3851.5</v>
+      </c>
+      <c r="C9" s="3">
+        <v>3678.9</v>
+      </c>
+      <c r="D9" s="3">
+        <v>3712.6</v>
+      </c>
+      <c r="E9" s="3">
+        <v>3764.9</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C10">
-        <v>3655.1</v>
-      </c>
-      <c r="D10">
-        <v>3707.1</v>
-      </c>
-      <c r="E10">
-        <v>3758.6</v>
+      <c r="B10" s="3">
+        <v>3860.8</v>
+      </c>
+      <c r="C10" s="3">
+        <v>3673.8</v>
+      </c>
+      <c r="D10" s="3">
+        <v>3709</v>
+      </c>
+      <c r="E10" s="3">
+        <v>3765.2</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D11">
-        <v>3671.4</v>
+      <c r="B11" s="3">
+        <v>3842.7</v>
+      </c>
+      <c r="C11" s="3">
+        <v>3663.1</v>
+      </c>
+      <c r="D11" s="3">
+        <v>3709</v>
+      </c>
+      <c r="E11" s="3">
+        <v>3763.2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="B12" s="3">
+        <v>3856.6</v>
+      </c>
+      <c r="C12" s="3">
+        <v>3671</v>
+      </c>
+      <c r="D12" s="3">
+        <v>3707.9</v>
+      </c>
+      <c r="E12" s="6">
+        <v>3764.9</v>
+      </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
@@ -1046,64 +1160,271 @@
       <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="12" t="s">
         <v>7</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="B15" s="3">
+        <v>4564.3999999999996</v>
+      </c>
+      <c r="C15" s="3">
+        <v>4898.3999999999996</v>
+      </c>
+      <c r="D15" s="3">
+        <v>4969</v>
+      </c>
+      <c r="E15" s="3">
+        <v>4909.8999999999996</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="14" t="s">
         <v>2</v>
       </c>
+      <c r="B16" s="3">
+        <v>5053.1000000000004</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4962</v>
+      </c>
       <c r="D16" s="3">
-        <v>5032.6000000000004</v>
+        <v>5043.3</v>
+      </c>
+      <c r="E16" s="3">
+        <v>4984.7</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C17" s="4">
-        <v>4959.8</v>
-      </c>
-      <c r="D17">
-        <v>5042.8</v>
-      </c>
-      <c r="E17">
-        <v>4984.6000000000004</v>
+      <c r="B17" s="3">
+        <v>5221</v>
+      </c>
+      <c r="C17" s="6">
+        <v>4962.1000000000004</v>
+      </c>
+      <c r="D17" s="3">
+        <v>5043.3999999999996</v>
+      </c>
+      <c r="E17" s="3">
+        <v>4983.3999999999996</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D18">
-        <v>5035.5</v>
-      </c>
-      <c r="E18" s="3"/>
+      <c r="B18" s="3">
+        <v>5192.5</v>
+      </c>
+      <c r="C18" s="3">
+        <v>4966.1000000000004</v>
+      </c>
+      <c r="D18" s="3">
+        <v>5046.3999999999996</v>
+      </c>
+      <c r="E18" s="3">
+        <v>4982.3</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="4"/>
+      <c r="B19" s="3">
+        <v>5171.3999999999996</v>
+      </c>
+      <c r="C19" s="3">
+        <v>4961.5</v>
+      </c>
+      <c r="D19" s="6">
+        <v>5047.8</v>
+      </c>
+      <c r="E19" s="3">
+        <v>4977.3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="B9:E9">
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
+    <cfRule type="colorScale" priority="34">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 B10:D10">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16 B17:D17">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 B11:E11 B10:D10">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16 B18:E18 B17:D17">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 B11:E12 B10:D10">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16 B19:D19 B18:E18 B17:D17">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:F4">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:F5">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:D19 B15:E18">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:E11">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:F5">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -1115,55 +1436,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B16:E16">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E16">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9 B10:D10">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E16 F14 B17:D17">
+  <conditionalFormatting sqref="B8:E12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:F5">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -1175,43 +1460,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9 B11:E11 B10:D10">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E16 B18:E18 B17:D17">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9 B11:E12 B10:D10">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E16 B18:E19 B17:D17">
+  <conditionalFormatting sqref="B4:F4">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:F5">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E19">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1223,68 +1496,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E4">
+  <conditionalFormatting sqref="B15:E19">
     <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:E5">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E19">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9:E11">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E5">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E12">
-    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1309,28 +1522,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1338,14 +1554,20 @@
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="3">
-        <v>1868</v>
+      <c r="B4">
+        <v>777.2</v>
       </c>
       <c r="C4" s="3">
-        <v>2689</v>
+        <v>1138.2</v>
       </c>
       <c r="D4" s="3">
-        <v>3412</v>
+        <v>1724.6</v>
+      </c>
+      <c r="E4" s="3">
+        <v>2333.6999999999998</v>
+      </c>
+      <c r="F4">
+        <v>2351.1999999999998</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1353,15 +1575,20 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>2148.3000000000002</v>
+        <v>847.1</v>
       </c>
       <c r="C5">
-        <v>3012.6</v>
-      </c>
-      <c r="D5">
-        <v>3943.1</v>
-      </c>
-      <c r="E5" s="4"/>
+        <v>1413.2</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1961</v>
+      </c>
+      <c r="E5" s="3">
+        <v>2817</v>
+      </c>
+      <c r="F5" s="4">
+        <v>2852.3</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
@@ -1373,10 +1600,10 @@
       <c r="C7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="11" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1384,42 +1611,86 @@
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B8" s="3">
+        <v>1663</v>
+      </c>
+      <c r="C8">
+        <v>2648.6</v>
+      </c>
+      <c r="D8">
+        <v>3915</v>
+      </c>
+      <c r="E8">
+        <v>3852.4</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="14" t="s">
         <v>2</v>
       </c>
+      <c r="B9">
+        <v>1673.2</v>
+      </c>
+      <c r="C9">
+        <v>2635.3</v>
+      </c>
       <c r="D9">
-        <v>5648.8</v>
+        <v>3860.7</v>
+      </c>
+      <c r="E9">
+        <v>4252.6000000000004</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="15" t="s">
         <v>3</v>
       </c>
+      <c r="B10">
+        <v>1665.8</v>
+      </c>
       <c r="C10">
-        <v>4886.8</v>
+        <v>2636.1</v>
       </c>
       <c r="D10">
-        <v>5644.2</v>
+        <v>3900.9</v>
       </c>
       <c r="E10">
-        <v>5655.1</v>
+        <v>4277.3</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B11">
+        <v>1682.6</v>
+      </c>
+      <c r="C11">
+        <v>2705.6</v>
+      </c>
       <c r="D11">
-        <v>5673.9</v>
+        <v>4019.8</v>
+      </c>
+      <c r="E11" s="3">
+        <v>4278</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="B12">
+        <v>1649.5</v>
+      </c>
+      <c r="C12">
+        <v>2662.1</v>
+      </c>
+      <c r="D12">
+        <v>3981.8</v>
+      </c>
+      <c r="E12" s="6">
+        <v>4223.2</v>
+      </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
@@ -1443,52 +1714,140 @@
       <c r="A15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="B15">
+        <v>1648.1</v>
+      </c>
+      <c r="C15" s="3">
+        <v>2624.1</v>
+      </c>
+      <c r="D15" s="3">
+        <v>3934</v>
+      </c>
+      <c r="E15" s="3">
+        <v>3750.1</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="14" t="s">
         <v>2</v>
       </c>
+      <c r="B16">
+        <v>1666.1</v>
+      </c>
+      <c r="C16">
+        <v>2619.4</v>
+      </c>
       <c r="D16" s="3">
-        <v>6675.1</v>
+        <v>3835.3</v>
+      </c>
+      <c r="E16">
+        <v>3901.4</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="15" t="s">
         <v>3</v>
       </c>
+      <c r="B17">
+        <v>1655.6</v>
+      </c>
       <c r="C17">
-        <v>4859.3</v>
+        <v>2626.7</v>
       </c>
       <c r="D17" s="3">
-        <v>7126.5</v>
-      </c>
-      <c r="E17" s="4">
-        <v>6681.1</v>
+        <v>3853.5</v>
+      </c>
+      <c r="E17" s="6">
+        <v>4032</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B18">
+        <v>1656.1</v>
+      </c>
+      <c r="C18" s="3">
+        <v>2629</v>
+      </c>
       <c r="D18" s="3">
-        <v>6922</v>
-      </c>
-      <c r="E18" s="3"/>
+        <v>3835.4</v>
+      </c>
+      <c r="E18" s="3">
+        <v>4085.5</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="4"/>
+      <c r="B19">
+        <v>1645.5</v>
+      </c>
+      <c r="C19">
+        <v>2579.6</v>
+      </c>
+      <c r="D19">
+        <v>3856.2</v>
+      </c>
+      <c r="E19" s="4">
+        <v>4103.5</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="B9:E9 C10">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 C10">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E10">
     <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
@@ -1500,7 +1859,550 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E17 F14">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E11">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E18">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E19">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:F4">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:F5">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:F5">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17:E17">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10:E10">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:E11">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16:E18">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:F4">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:F5">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>1378.2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2043.1</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2859.1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>3629.1</v>
+      </c>
+      <c r="F4" s="6">
+        <v>3443.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>1441.6</v>
+      </c>
+      <c r="C5">
+        <v>2154.9</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3050.5</v>
+      </c>
+      <c r="E5" s="3">
+        <v>3952.2</v>
+      </c>
+      <c r="F5" s="6">
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>2996.7</v>
+      </c>
+      <c r="C8">
+        <v>4863.8999999999996</v>
+      </c>
+      <c r="D8">
+        <v>5746.5</v>
+      </c>
+      <c r="E8">
+        <v>5729.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <v>3009.4</v>
+      </c>
+      <c r="C9">
+        <v>4759.2</v>
+      </c>
+      <c r="D9">
+        <v>5614.8</v>
+      </c>
+      <c r="E9" s="4">
+        <v>5566.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="4">
+        <v>3010.8</v>
+      </c>
+      <c r="C10">
+        <v>4916.8999999999996</v>
+      </c>
+      <c r="D10">
+        <v>5593.1</v>
+      </c>
+      <c r="E10" s="6">
+        <v>5556</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="4">
+        <v>3050.8</v>
+      </c>
+      <c r="C11" s="3">
+        <v>4770</v>
+      </c>
+      <c r="D11">
+        <v>5628</v>
+      </c>
+      <c r="E11" s="4">
+        <v>5615.3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>3000.3</v>
+      </c>
+      <c r="C12" s="3">
+        <v>4983</v>
+      </c>
+      <c r="D12">
+        <v>5631.3</v>
+      </c>
+      <c r="E12" s="6">
+        <v>5536.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>2988.3</v>
+      </c>
+      <c r="C15" s="3">
+        <v>4910.3</v>
+      </c>
+      <c r="D15" s="3">
+        <v>7107.2</v>
+      </c>
+      <c r="E15" s="3">
+        <v>7081.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16">
+        <v>3023.9</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4915</v>
+      </c>
+      <c r="D16" s="3">
+        <v>6953</v>
+      </c>
+      <c r="E16" s="3">
+        <v>7207</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17">
+        <v>2957.7</v>
+      </c>
+      <c r="C17">
+        <v>4937.8999999999996</v>
+      </c>
+      <c r="D17" s="3">
+        <v>6779.1</v>
+      </c>
+      <c r="E17" s="4">
+        <v>7200.9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18">
+        <v>3018.9</v>
+      </c>
+      <c r="C18">
+        <v>4990.8999999999996</v>
+      </c>
+      <c r="D18" s="3">
+        <v>7176</v>
+      </c>
+      <c r="E18" s="3">
+        <v>6833.6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19">
+        <v>2987.7</v>
+      </c>
+      <c r="C19">
+        <v>4981.8</v>
+      </c>
+      <c r="D19" s="3">
+        <v>7183</v>
+      </c>
+      <c r="E19" s="4">
+        <v>7104.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9:E9 C10">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B16:E16">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E9 C10">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E10">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E17 F14">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:E11">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E18">
     <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
@@ -1512,31 +2414,55 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9 C10">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E16">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E10">
+  <conditionalFormatting sqref="B8:E12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E19">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:F4">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:F5">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:F5">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -1548,31 +2474,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E17 F14">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E11">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E18">
+  <conditionalFormatting sqref="C17:E17">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -1584,19 +2486,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E12">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E19">
+  <conditionalFormatting sqref="C10:E10">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1608,7 +2498,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E4">
+  <conditionalFormatting sqref="C9:E11">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16:E18">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:F4">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -1620,7 +2534,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:E5">
+  <conditionalFormatting sqref="B5:F5">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -1632,56 +2546,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E5">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C17:E17">
+  <conditionalFormatting sqref="B8:E9">
     <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C10:E10">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9:E11">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C16:E18">
-    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>